<commit_message>
Implement index for every field
</commit_message>
<xml_diff>
--- a/BD.xlsx
+++ b/BD.xlsx
@@ -8,12 +8,17 @@
   <sheets>
     <sheet name="Libros" r:id="rId3" sheetId="1"/>
     <sheet name="Indice" r:id="rId4" sheetId="2"/>
+    <sheet name="Indice_Nombre" r:id="rId5" sheetId="3"/>
+    <sheet name="Indice_Autor" r:id="rId6" sheetId="4"/>
+    <sheet name="Indice_Editorial" r:id="rId7" sheetId="5"/>
+    <sheet name="Indice_Anio" r:id="rId8" sheetId="6"/>
+    <sheet name="Indice_Ubicacion" r:id="rId9" sheetId="7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="86">
   <si>
     <t>ID</t>
   </si>
@@ -217,6 +222,60 @@
   </si>
   <si>
     <t>Estante A4</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>asasa</t>
+  </si>
+  <si>
+    <t>asas</t>
+  </si>
+  <si>
+    <t>dsdfdf</t>
+  </si>
+  <si>
+    <t>1701</t>
+  </si>
+  <si>
+    <t>fsdfd</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>Clave(Nombre)</t>
+  </si>
+  <si>
+    <t>Clave(Autor)</t>
+  </si>
+  <si>
+    <t>Clave(Editorial)</t>
+  </si>
+  <si>
+    <t>Clave(Año)</t>
+  </si>
+  <si>
+    <t>Clave(Ubicación)</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>DEL RAYE A LA RUTINA</t>
+  </si>
+  <si>
+    <t>GONZALO VALDERRAMA</t>
+  </si>
+  <si>
+    <t>PLANETA</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>ESTANTE D9</t>
   </si>
 </sst>
 </file>
@@ -261,7 +320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -484,6 +543,26 @@
         <v>67</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -491,7 +570,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -582,6 +661,144 @@
         <v>5.0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B12" t="n" s="0">
+        <v>11.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="B2" t="n" s="0">
+        <v>11.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="B2" t="n" s="0">
+        <v>11.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="B2" t="n" s="0">
+        <v>11.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="B2" t="n" s="0">
+        <v>11.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B2" t="n" s="0">
+        <v>11.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>